<commit_message>
06 10 26 v8
</commit_message>
<xml_diff>
--- a/Tabelas Especificas/TabelaB-V2.xlsx
+++ b/Tabelas Especificas/TabelaB-V2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PainelNovo\Tabelas Especificas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC8CEDDE-52EA-4F11-89A7-4FE8A98608D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46510498-A96A-4B71-986A-2FC133EF91A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="918" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="918" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contrato" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5606" uniqueCount="1330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5612" uniqueCount="1331">
   <si>
     <t>Contrato</t>
   </si>
@@ -4046,6 +4046,9 @@
   </si>
   <si>
     <t>Dia da Consciência Negra</t>
+  </si>
+  <si>
+    <t>2026#08</t>
   </si>
 </sst>
 </file>
@@ -4299,86 +4302,6 @@
   </cellStyles>
   <dxfs count="85">
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="9" tint="0.79998168889431442"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ \(ddd\)"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <strike/>
         <u/>
@@ -4520,6 +4443,86 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="9" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ \(ddd\)"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="9" tint="0.79998168889431442"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -5140,59 +5143,59 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A3BD3951-8AEF-44AE-85E4-BF63B4B4FE00}" name="CalendarioFeriado" displayName="CalendarioFeriado" ref="A1:E81" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A3BD3951-8AEF-44AE-85E4-BF63B4B4FE00}" name="CalendarioFeriado" displayName="CalendarioFeriado" ref="A1:E81" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="A1:E81" xr:uid="{A3BD3951-8AEF-44AE-85E4-BF63B4B4FE00}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F8E60F0F-82D7-4C55-8668-7E14F02548C1}" name="Data" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{E6072DB0-915C-4537-BA4D-27E948186672}" name="Feriado" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{0A01562B-D7CD-45AB-8FD2-CFC786839537}" name="Abrangência" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{8106E8D7-6B09-48AD-A249-8693D616B525}" name="Tipo" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{D9E5C778-1EBD-4197-B8B0-5F8039877089}" name="UF" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{F8E60F0F-82D7-4C55-8668-7E14F02548C1}" name="Data" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{E6072DB0-915C-4537-BA4D-27E948186672}" name="Feriado" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{0A01562B-D7CD-45AB-8FD2-CFC786839537}" name="Abrangência" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{8106E8D7-6B09-48AD-A249-8693D616B525}" name="Tipo" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{D9E5C778-1EBD-4197-B8B0-5F8039877089}" name="UF" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{47969D70-6C9C-4F7C-9138-C79BEA291514}" name="Estrutura" displayName="Estrutura" ref="A1:D94" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{47969D70-6C9C-4F7C-9138-C79BEA291514}" name="Estrutura" displayName="Estrutura" ref="A1:D94" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:D94" xr:uid="{47969D70-6C9C-4F7C-9138-C79BEA291514}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{5CFB21F2-08F8-4150-AF24-3290D1FA81D0}" name="Lotação" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{EC3BEFCE-97FF-4352-B70E-0CB66847395C}" name="Diretoria Executiva" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{039770E2-404B-4FC2-8669-39177A750314}" name="Gerência Executiva" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{D6922F5E-C416-4DFD-9483-94847F7B7982}" name="Ativo" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{5CFB21F2-08F8-4150-AF24-3290D1FA81D0}" name="Lotação" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{EC3BEFCE-97FF-4352-B70E-0CB66847395C}" name="Diretoria Executiva" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{039770E2-404B-4FC2-8669-39177A750314}" name="Gerência Executiva" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{D6922F5E-C416-4DFD-9483-94847F7B7982}" name="Ativo" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9D46CC66-4E2E-4265-9334-E5D69C3C90F4}" name="Grupo" displayName="Grupo" ref="A1:F394" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9D46CC66-4E2E-4265-9334-E5D69C3C90F4}" name="Grupo" displayName="Grupo" ref="A1:F394" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A1:F394" xr:uid="{9D46CC66-4E2E-4265-9334-E5D69C3C90F4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F394">
     <sortCondition ref="E1:E394"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{3D8FF589-B5E4-4801-A959-475795493EB8}" name="Município" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{881028AA-7608-4AB6-A013-8346CD659EBA}" name="UF" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{9B7D3AF5-7A2E-4DCE-9F7E-BC89DFC1F456}" name="RMT" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{2E44873E-7890-4462-8DD1-6C82AAC0D6BE}" name="Região" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{03A237A3-A7BD-423E-AD26-C76AF057C7EE}" name="Grupo" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{6785FF19-9D6F-4D1F-A12F-CA56CAE3EBB4}" name="Contrato" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{3D8FF589-B5E4-4801-A959-475795493EB8}" name="Município" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{881028AA-7608-4AB6-A013-8346CD659EBA}" name="UF" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{9B7D3AF5-7A2E-4DCE-9F7E-BC89DFC1F456}" name="RMT" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{2E44873E-7890-4462-8DD1-6C82AAC0D6BE}" name="Região" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{03A237A3-A7BD-423E-AD26-C76AF057C7EE}" name="Grupo" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{6785FF19-9D6F-4D1F-A12F-CA56CAE3EBB4}" name="Contrato" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}" name="FDM_IAPFARQ" displayName="FDM_IAPFARQ" ref="A1:E25" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
-  <autoFilter ref="A1:E25" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}" name="FDM_IAPFARQ" displayName="FDM_IAPFARQ" ref="A1:E28" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E28" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8441FCBE-E45F-4BE2-B9F9-1923EE72D293}" name="Medição" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{1B8ACFB0-E0FB-4FAA-9742-75748BC308D0}" name="Contrato" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{C27C6068-3982-4FCE-A96C-C250BC27EAAF}" name="Item contrato" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{0832F87C-BEC8-4F26-AF6D-726FC6CFF5D9}" name="IAPFARQ (%)" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{08B9E89A-8CAB-4E87-8C5C-3D57B4E1A7A5}" name="FDM" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{8441FCBE-E45F-4BE2-B9F9-1923EE72D293}" name="Medição" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{1B8ACFB0-E0FB-4FAA-9742-75748BC308D0}" name="Contrato" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{C27C6068-3982-4FCE-A96C-C250BC27EAAF}" name="Item contrato" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{0832F87C-BEC8-4F26-AF6D-726FC6CFF5D9}" name="IAPFARQ (%)" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{08B9E89A-8CAB-4E87-8C5C-3D57B4E1A7A5}" name="FDM" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12549,10 +12552,10 @@
     <sortCondition ref="A2:A108"/>
   </sortState>
   <conditionalFormatting sqref="A2:A184">
-    <cfRule type="duplicateValues" dxfId="8" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:A38">
-    <cfRule type="expression" dxfId="7" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
       <formula>AND(#REF!&lt;2,#REF!=1)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -28595,18 +28598,69 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>1315</v>
+        <v>1330</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>1264</v>
+      </c>
+      <c r="C25" s="1">
+        <v>1</v>
+      </c>
+      <c r="D25" s="1">
+        <v>56.29</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>1264</v>
+      </c>
+      <c r="C26" s="1">
+        <v>2</v>
+      </c>
+      <c r="D26" s="1">
+        <v>77.36</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>1258</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C27" s="1">
+        <v>1</v>
+      </c>
+      <c r="D27" s="1">
+        <v>23.08</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="C28" s="1">
         <v>2</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D28" s="1">
         <v>80</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E28" s="1">
         <v>0.97</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v8 22 10 2026
</commit_message>
<xml_diff>
--- a/Tabelas Especificas/TabelaB-V2.xlsx
+++ b/Tabelas Especificas/TabelaB-V2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PainelNovo\Tabelas Especificas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46510498-A96A-4B71-986A-2FC133EF91A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3278991-7587-4402-92FB-9E5150060EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="918" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Calendario!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Centro'!$A$1:$H$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">FDM_IAPFARQ!$A$1:$H$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">FDM_IAPFARQ!$A$1:$H$204</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Grupo!$A$1:$F$394</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Localidade!$A$1:$B$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Origem_Destino!$A$1:$Q$73</definedName>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5612" uniqueCount="1331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5620" uniqueCount="1332">
   <si>
     <t>Contrato</t>
   </si>
@@ -4049,6 +4049,9 @@
   </si>
   <si>
     <t>2026#08</t>
+  </si>
+  <si>
+    <t>2026#09</t>
   </si>
 </sst>
 </file>
@@ -5188,8 +5191,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}" name="FDM_IAPFARQ" displayName="FDM_IAPFARQ" ref="A1:E28" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E28" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}" name="FDM_IAPFARQ" displayName="FDM_IAPFARQ" ref="A1:E32" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E32" xr:uid="{44E4EBDF-4B50-404B-8A95-71C77FDCE640}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{8441FCBE-E45F-4BE2-B9F9-1923EE72D293}" name="Medição" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{1B8ACFB0-E0FB-4FAA-9742-75748BC308D0}" name="Contrato" dataDxfId="5"/>
@@ -28182,7 +28185,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr codeName="Planilha10"/>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr defaultColWidth="23.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="23.109375" style="1"/>
@@ -28607,10 +28610,10 @@
         <v>1</v>
       </c>
       <c r="D25" s="1">
-        <v>56.29</v>
+        <v>100</v>
       </c>
       <c r="E25" s="1">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -28624,10 +28627,10 @@
         <v>2</v>
       </c>
       <c r="D26" s="1">
-        <v>77.36</v>
+        <v>100</v>
       </c>
       <c r="E26" s="1">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -28641,10 +28644,10 @@
         <v>1</v>
       </c>
       <c r="D27" s="1">
-        <v>23.08</v>
+        <v>100</v>
       </c>
       <c r="E27" s="1">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -28658,18 +28661,89 @@
         <v>2</v>
       </c>
       <c r="D28" s="1">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="E28" s="1">
-        <v>0.97</v>
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>1264</v>
+      </c>
+      <c r="C29" s="1">
+        <v>1</v>
+      </c>
+      <c r="D29" s="1">
+        <v>100</v>
+      </c>
+      <c r="E29" s="1">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>1264</v>
+      </c>
+      <c r="C30" s="1">
+        <v>2</v>
+      </c>
+      <c r="D30" s="1">
+        <v>100</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="C31" s="1">
+        <v>1</v>
+      </c>
+      <c r="D31" s="1">
+        <v>100</v>
+      </c>
+      <c r="E31" s="1">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="C32" s="1">
+        <v>2</v>
+      </c>
+      <c r="D32" s="1">
+        <v>100</v>
+      </c>
+      <c r="E32" s="1">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="84" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D84" s="12"/>
+      <c r="E84" s="12"/>
+      <c r="H84" s="13" t="s">
+        <v>1185</v>
       </c>
     </row>
     <row r="85" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D85" s="12"/>
-      <c r="E85" s="12"/>
-      <c r="H85" s="13" t="s">
-        <v>1185</v>
-      </c>
+      <c r="H85" s="14"/>
     </row>
     <row r="86" spans="4:8" x14ac:dyDescent="0.3">
       <c r="H86" s="14"/>
@@ -28678,55 +28752,52 @@
       <c r="H87" s="14"/>
     </row>
     <row r="88" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="H88" s="14"/>
+      <c r="E88" s="12"/>
+      <c r="H88" s="13"/>
     </row>
     <row r="89" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D89" s="12"/>
       <c r="E89" s="12"/>
-      <c r="H89" s="13"/>
+      <c r="H89" s="13" t="s">
+        <v>1186</v>
+      </c>
     </row>
     <row r="90" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D90" s="12"/>
       <c r="E90" s="12"/>
       <c r="H90" s="13" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="91" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D91" s="12"/>
       <c r="E91" s="12"/>
       <c r="H91" s="13" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="92" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D92" s="12"/>
       <c r="E92" s="12"/>
       <c r="H92" s="13" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="93" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D93" s="12"/>
-      <c r="E93" s="12"/>
       <c r="H93" s="13" t="s">
-        <v>1189</v>
-      </c>
-    </row>
-    <row r="94" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D94" s="12"/>
-      <c r="H94" s="13" t="s">
         <v>1190</v>
+      </c>
+    </row>
+    <row r="95" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="E95" s="12"/>
+      <c r="H95" s="13" t="s">
+        <v>1192</v>
       </c>
     </row>
     <row r="96" spans="4:8" x14ac:dyDescent="0.3">
       <c r="E96" s="12"/>
       <c r="H96" s="13" t="s">
-        <v>1192</v>
-      </c>
-    </row>
-    <row r="97" spans="5:8" x14ac:dyDescent="0.3">
-      <c r="E97" s="12"/>
-      <c r="H97" s="13" t="s">
         <v>1191</v>
       </c>
     </row>

</xml_diff>